<commit_message>
Junior IT-Jobs quellennah - 11 Jobs (+11)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Quellennah.xlsx
+++ b/download/Junior_IT_Jobs_Quellennah.xlsx
@@ -449,8 +449,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:AI12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -2232,6 +2232,151 @@
       </c>
       <c r="AI11" s="2" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Q-00011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>IKS-Network–Operation-Service</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iks-network.com/leistungen/it-services/iks-managed-services#os</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>IKS GmbH - pure IT-Dienstleistungen</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iks-network.com</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iks-network.com/ueber-die-iks-mobile/iks-karriere</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>Dienstleistung</t>
+        </is>
+      </c>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>Website: https://www.iks-network.com</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr"/>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr"/>
+      <c r="AD12" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 17:46:04</t>
+        </is>
+      </c>
+      <c r="AF12" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG12" s="2" t="inlineStr">
+        <is>
+          <t>58f5416b91e6</t>
+        </is>
+      </c>
+      <c r="AH12" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/IKS GmbH - pure IT-Dienstleistungen_career.html</t>
+        </is>
+      </c>
+      <c r="AI12" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Junior IT-Jobs quellennah - 12 Jobs (+12)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Quellennah.xlsx
+++ b/download/Junior_IT_Jobs_Quellennah.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI12"/>
+  <dimension ref="A1:AI13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2377,6 +2377,151 @@
       </c>
       <c r="AI12" s="2" t="inlineStr"/>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Q-00012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>IKS-Network–Visibility-Service</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iks-network.com/leistungen/it-services/iks-managed-services#vs</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>IKS GmbH - pure IT-Dienstleistungen</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iks-network.com</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iks-network.com/ueber-die-iks-mobile/iks-karriere</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>Dienstleistung</t>
+        </is>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>Website: https://www.iks-network.com</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr"/>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr"/>
+      <c r="AD13" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE13" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 17:46:07</t>
+        </is>
+      </c>
+      <c r="AF13" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG13" s="2" t="inlineStr">
+        <is>
+          <t>58f5416b91e6</t>
+        </is>
+      </c>
+      <c r="AH13" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/IKS GmbH - pure IT-Dienstleistungen_career.html</t>
+        </is>
+      </c>
+      <c r="AI13" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Junior IT-Jobs quellennah - 13 Jobs (+13)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Quellennah.xlsx
+++ b/download/Junior_IT_Jobs_Quellennah.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI13"/>
+  <dimension ref="A1:AI14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2522,6 +2522,151 @@
       </c>
       <c r="AI13" s="2" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Q-00013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>www.iks-network.com/downloads/Infopflicht-Bewerber.pdf</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iks-network.com/downloads/Infopflicht-Bewerber.pdf</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>IKS GmbH - pure IT-Dienstleistungen</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iks-network.com</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iks-network.com/ueber-die-iks-mobile/iks-karriere</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>Dienstleistung</t>
+        </is>
+      </c>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>Website: https://www.iks-network.com</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr"/>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr"/>
+      <c r="AD14" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 17:46:09</t>
+        </is>
+      </c>
+      <c r="AF14" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG14" s="2" t="inlineStr">
+        <is>
+          <t>58f5416b91e6</t>
+        </is>
+      </c>
+      <c r="AH14" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/IKS GmbH - pure IT-Dienstleistungen_career.html</t>
+        </is>
+      </c>
+      <c r="AI14" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Junior IT-Jobs quellennah - 14 Jobs (+14)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Quellennah.xlsx
+++ b/download/Junior_IT_Jobs_Quellennah.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI14"/>
+  <dimension ref="A1:AI15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2667,6 +2667,151 @@
       </c>
       <c r="AI14" s="2" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Q-00014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>info@iks-network.com</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>mailto:info@iks-network.com</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>IKS GmbH - pure IT-Dienstleistungen</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iks-network.com</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.iks-network.com/ueber-die-iks-mobile/iks-karriere</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>Dienstleistung</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>Website: https://www.iks-network.com</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr"/>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr"/>
+      <c r="AD15" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 17:46:11</t>
+        </is>
+      </c>
+      <c r="AF15" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG15" s="2" t="inlineStr">
+        <is>
+          <t>58f5416b91e6</t>
+        </is>
+      </c>
+      <c r="AH15" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/IKS GmbH - pure IT-Dienstleistungen_career.html</t>
+        </is>
+      </c>
+      <c r="AI15" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Junior IT-Jobs quellennah - 20 Jobs (+12)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Quellennah.xlsx
+++ b/download/Junior_IT_Jobs_Quellennah.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI5"/>
+  <dimension ref="A1:AI21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1254,6 +1254,2317 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Q-00005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Embedded Softwareentwickler C++ (m/w/d) in Vollzeit, unbefristeter Vertrag</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Softwareentwicklung</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.afra.de/jobs</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>AFRA Anwenderfreundliche Automatisierung GmbH</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.afra.de/</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.afra.de/jobs</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>url_pattern: AFRA Anwenderfreundliche Automatisierung GmbH</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE6" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:42:17</t>
+        </is>
+      </c>
+      <c r="AF6" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG6" s="2" t="inlineStr">
+        <is>
+          <t>030562449bdb</t>
+        </is>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/AFRA Anwenderfreundliche Automatisierung GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Q-00006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Software Support Spezialist – DACH und Osteuropa</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.aiscorp.com/de/ueber-uns/karriere/</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Aegis Software GmbH</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.aiscorp.com/de/</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.aiscorp.com/de/ueber-uns/karriere/</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Aegis Software GmbH</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y7" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z7" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE7" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:42:24</t>
+        </is>
+      </c>
+      <c r="AF7" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG7" s="2" t="inlineStr">
+        <is>
+          <t>86a487236c9d</t>
+        </is>
+      </c>
+      <c r="AH7" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Aegis Software GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Q-00007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Algorithmus Entwickler</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Softwareentwicklung</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.algorithmus-schmiede.de/karriere/</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>Algorithmus Schmiede</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.algorithmus-schmiede.de/</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.algorithmus-schmiede.de/karriere/</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Algorithmus Schmiede</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="inlineStr"/>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr">
+        <is>
+          <t>entwickler</t>
+        </is>
+      </c>
+      <c r="Z8" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr"/>
+      <c r="AD8" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:42:31</t>
+        </is>
+      </c>
+      <c r="AF8" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG8" s="2" t="inlineStr">
+        <is>
+          <t>9840912c7879</t>
+        </is>
+      </c>
+      <c r="AH8" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Algorithmus Schmiede_career.html</t>
+        </is>
+      </c>
+      <c r="AI8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Q-00008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Sie entwerfen Schnittstellen, konzipieren Services, entwickeln Testkonzepte dazu und setzen das in realen Code um.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.clearsystems.de/de/karriere</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>CLEAR IT GmbH</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.clearsystems.de</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.clearsystems.de/de/karriere</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: CLEAR IT GmbH</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="inlineStr"/>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="Z9" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB9" s="2" t="inlineStr"/>
+      <c r="AC9" s="2" t="inlineStr"/>
+      <c r="AD9" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE9" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:43:45</t>
+        </is>
+      </c>
+      <c r="AF9" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG9" s="2" t="inlineStr">
+        <is>
+          <t>d670446e12c1</t>
+        </is>
+      </c>
+      <c r="AH9" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/CLEAR IT GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Q-00009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Ehrlichkeit, Flexibilität und direkte Kommunikation schaffen für uns die ideale Umgebung für persönliches Wachstum und erstklassige Team-Ergebnisse. Werde jetzt Teil des Hansefit-Teams und revolutioniere mit uns die Zukunft von Firmenfitness.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>https://hansefit.de/karriere/</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>City Fitness Erlangen</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>https://hansefit.de/de/studio-finden/erlangen/fitnessstudio/city-fitness-erlangen/</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>https://hansefit.de/karriere/</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>Fitness</t>
+        </is>
+      </c>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: City Fitness Erlangen</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr"/>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>it-</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr"/>
+      <c r="AD10" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:44:19</t>
+        </is>
+      </c>
+      <c r="AF10" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG10" s="2" t="inlineStr">
+        <is>
+          <t>d637bb97321b</t>
+        </is>
+      </c>
+      <c r="AH10" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/City Fitness Erlangen_career.html</t>
+        </is>
+      </c>
+      <c r="AI10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Q-00010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>HR &amp; Administration</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Systemadministration</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>https://cognitionteam.com/company/careers</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>Cognitionteam</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>https://cognitionteam.com/</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>https://cognitionteam.com/company/careers</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Cognitionteam</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr"/>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr"/>
+      <c r="AD11" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE11" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:44:25</t>
+        </is>
+      </c>
+      <c r="AF11" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG11" s="2" t="inlineStr">
+        <is>
+          <t>f281e11dfc4d</t>
+        </is>
+      </c>
+      <c r="AH11" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Cognitionteam_career.html</t>
+        </is>
+      </c>
+      <c r="AI11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Q-00011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Application re-Engineering</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>https://cognitionteam.com/company/engineering/application-re-engineering</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>Cognitionteam</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>https://cognitionteam.com/</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>https://cognitionteam.com/company/careers</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Cognitionteam</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr"/>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr"/>
+      <c r="AD12" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:44:25</t>
+        </is>
+      </c>
+      <c r="AF12" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG12" s="2" t="inlineStr">
+        <is>
+          <t>f281e11dfc4d</t>
+        </is>
+      </c>
+      <c r="AH12" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Cognitionteam_career.html</t>
+        </is>
+      </c>
+      <c r="AI12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Q-00012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>INNENARCHITEKT*IN/PLANER*IN (M/W/D)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>https://dreyer-gmbh.de/jobs/</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Dreyer Haustechnik GmbH</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>https://dreyer-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>https://dreyer-gmbh.de/jobs/</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Dreyer Haustechnik GmbH</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr"/>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>architekt</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr"/>
+      <c r="AD13" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE13" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:44:47</t>
+        </is>
+      </c>
+      <c r="AF13" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG13" s="2" t="inlineStr">
+        <is>
+          <t>7625335a6ee3</t>
+        </is>
+      </c>
+      <c r="AH13" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Dreyer Haustechnik GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Q-00013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Support the coordination and administration of international licensing partnerships</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Systemadministration</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>https://giants-software.com/career.php</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>GIANTS Software Entertainment GmbH</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>https://giants-software.com/contact.php</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>https://giants-software.com/career.php</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: GIANTS Software Entertainment GmbH</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr"/>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>intern</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr"/>
+      <c r="AD14" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:45:28</t>
+        </is>
+      </c>
+      <c r="AF14" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG14" s="2" t="inlineStr">
+        <is>
+          <t>5b111c02b887</t>
+        </is>
+      </c>
+      <c r="AH14" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/GIANTS Software Entertainment GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Q-00014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>„Als Webentwickler der Spedition und meine Tätigkeit als Ausbilder für drei IT-Berufe, ist mein Arbeitsalltag geprägt von Abwechslung, Spaß und Spannung!“</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Softwareentwicklung</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>https://geis-group.eu/karriere</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>Geis Eurocargo Erlangen-Frauenaurach</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>https://geis-group.eu</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>https://geis-group.eu/karriere</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>spedition</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Geis Eurocargo Erlangen-Frauenaurach</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr"/>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>entwickler</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr"/>
+      <c r="AD15" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:45:53</t>
+        </is>
+      </c>
+      <c r="AF15" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG15" s="2" t="inlineStr">
+        <is>
+          <t>4b814a183300</t>
+        </is>
+      </c>
+      <c r="AH15" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Geis Eurocargo Erlangen-Frauenaurach_career.html</t>
+        </is>
+      </c>
+      <c r="AI15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Q-00015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineering</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Softwareentwicklung</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.heitec.de/karriere</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>HEITEC AG - Erlangen</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.heitec.de/ueber-heitec/standorte/deutschland/erlangen</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.heitec.de/karriere</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: HEITEC AG - Erlangen</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr"/>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr"/>
+      <c r="AD16" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:46:34</t>
+        </is>
+      </c>
+      <c r="AF16" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG16" s="2" t="inlineStr">
+        <is>
+          <t>4fa067f9df18</t>
+        </is>
+      </c>
+      <c r="AH16" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/HEITEC AG - Erlangen_career.html</t>
+        </is>
+      </c>
+      <c r="AI16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Q-00016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Digitales Engineering</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Startseite
+Leistungen
+Digitalisierung
+Digitales Engineering
+Schnell. Durchgängig. Sicher.
+Mit dem Einsatz von digitalen Technologien und Werkzeugen, verkürzen wir Ihren Entwicklungsprozess, erfüllen höchste Qualitätsansprüche und steigern ihre Produktivität. Unsere Methoden ermöglichen Interoperabilität über alle Phasen ihres Product Lifecycles und sind auf die Steigerung ihrer Wertschöpfung ausgerichtet.
+Wir erstellen für Sie Simulationsmodelle zur Planung und Inbetriebnahme von Maschinen und Anlagen im Brown- und Greenfield. Unser langjähriges Know-how, generische und spezialisierte Bibliotheken, wie auch der Einsatz von unterschiedlichen Simulationstools ermöglich uns eine effiziente Umsetzung.
+Digitale Zukunft
+Der Einsatz von digitalen Technologien ist der Türöffner für wirtschaftlichen Erfolg in der Zukunft. Lassen Sie uns den Weg gemeinsam beschreiten!
+Michael Reinke | Abteilungsleiter Digitales Engineering
+Accelerator für Ihre digitale Planung
+In der Planung setzen wir uns</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.heitec.de/leistungen/digitalisierung/digital-engineering</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>HEITEC AG - Erlangen</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.heitec.de/ueber-heitec/standorte/deutschland/erlangen</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.heitec.de/karriere</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: HEITEC AG - Erlangen</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr"/>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr"/>
+      <c r="AC17" s="2" t="inlineStr"/>
+      <c r="AD17" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:46:34</t>
+        </is>
+      </c>
+      <c r="AF17" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG17" s="2" t="inlineStr">
+        <is>
+          <t>4fa067f9df18</t>
+        </is>
+      </c>
+      <c r="AH17" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/HEITEC AG - Erlangen_career.html</t>
+        </is>
+      </c>
+      <c r="AI17" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/job_detail_v3/job_58139.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Q-00017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Trainer Real-Time (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inchron.com/careers/</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>INCHRON AG</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inchron.com/</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inchron.com/careers/</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: INCHRON AG</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="inlineStr"/>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z18" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA18" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB18" s="2" t="inlineStr"/>
+      <c r="AC18" s="2" t="inlineStr"/>
+      <c r="AD18" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:47:00</t>
+        </is>
+      </c>
+      <c r="AF18" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG18" s="2" t="inlineStr">
+        <is>
+          <t>0f26da73b2a5</t>
+        </is>
+      </c>
+      <c r="AH18" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/INCHRON AG_career.html</t>
+        </is>
+      </c>
+      <c r="AI18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Q-00018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Event Chain Engineering</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inchron.com/event-chain-engineering/</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr"/>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>INCHRON AG</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inchron.com/</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inchron.com/careers/</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: INCHRON AG</t>
+        </is>
+      </c>
+      <c r="W19" s="2" t="inlineStr"/>
+      <c r="X19" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y19" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z19" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA19" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB19" s="2" t="inlineStr"/>
+      <c r="AC19" s="2" t="inlineStr"/>
+      <c r="AD19" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:47:00</t>
+        </is>
+      </c>
+      <c r="AF19" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG19" s="2" t="inlineStr">
+        <is>
+          <t>0f26da73b2a5</t>
+        </is>
+      </c>
+      <c r="AH19" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/INCHRON AG_career.html</t>
+        </is>
+      </c>
+      <c r="AI19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Q-00019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Requirements Engineering</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>UX/UI Design</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inchron.com/requirements-engineering-service/</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>INCHRON AG</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inchron.com/</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inchron.com/careers/</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: INCHRON AG</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="inlineStr"/>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA20" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="inlineStr"/>
+      <c r="AD20" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:47:00</t>
+        </is>
+      </c>
+      <c r="AF20" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG20" s="2" t="inlineStr">
+        <is>
+          <t>0f26da73b2a5</t>
+        </is>
+      </c>
+      <c r="AH20" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/INCHRON AG_career.html</t>
+        </is>
+      </c>
+      <c r="AI20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Q-00020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Customer Support Login</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inchron.com/supportlogin/</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>INCHRON AG</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inchron.com/</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.inchron.com/careers/</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U21" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: INCHRON AG</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="inlineStr"/>
+      <c r="X21" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y21" s="2" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="Z21" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA21" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB21" s="2" t="inlineStr"/>
+      <c r="AC21" s="2" t="inlineStr"/>
+      <c r="AD21" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:47:00</t>
+        </is>
+      </c>
+      <c r="AF21" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG21" s="2" t="inlineStr">
+        <is>
+          <t>0f26da73b2a5</t>
+        </is>
+      </c>
+      <c r="AH21" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/INCHRON AG_career.html</t>
+        </is>
+      </c>
+      <c r="AI21" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Junior IT-Jobs quellennah - 24 Jobs (+10)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Quellennah.xlsx
+++ b/download/Junior_IT_Jobs_Quellennah.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI21"/>
+  <dimension ref="A1:AI25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="AE16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 18:46:34</t>
+          <t>2026-05-14 18:46:38</t>
         </is>
       </c>
       <c r="AF16" s="2" t="inlineStr">
@@ -2961,7 +2961,7 @@
       </c>
       <c r="AE17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 18:46:34</t>
+          <t>2026-05-14 18:46:38</t>
         </is>
       </c>
       <c r="AF17" s="2" t="inlineStr">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="AI17" s="2" t="inlineStr">
         <is>
-          <t>/home/z/my-project/download/job_detail_v3/job_58139.html</t>
+          <t>/home/z/my-project/download/job_detail_v3/job_86349.html</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3110,7 @@
       </c>
       <c r="AE18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 18:47:00</t>
+          <t>2026-05-14 18:47:05</t>
         </is>
       </c>
       <c r="AF18" s="2" t="inlineStr">
@@ -3255,7 +3255,7 @@
       </c>
       <c r="AE19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 18:47:00</t>
+          <t>2026-05-14 18:47:05</t>
         </is>
       </c>
       <c r="AF19" s="2" t="inlineStr">
@@ -3400,7 +3400,7 @@
       </c>
       <c r="AE20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 18:47:00</t>
+          <t>2026-05-14 18:47:05</t>
         </is>
       </c>
       <c r="AF20" s="2" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="AE21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 18:47:00</t>
+          <t>2026-05-14 18:47:05</t>
         </is>
       </c>
       <c r="AF21" s="2" t="inlineStr">
@@ -3564,6 +3564,590 @@
         </is>
       </c>
       <c r="AI21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Q-00021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>CFD, Engineering und Consulting</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>https://invent-uv.de/jobs-karriere/arbeiten-bei-invent/</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr"/>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>INVENT Umwelt- und Verfahrenstechnik AG</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>https://invent-uv.de</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>https://invent-uv.de/jobs-karriere/arbeiten-bei-invent/</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>Maschinenbau</t>
+        </is>
+      </c>
+      <c r="T22" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: INVENT Umwelt- und Verfahrenstechnik AG</t>
+        </is>
+      </c>
+      <c r="W22" s="2" t="inlineStr"/>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y22" s="2" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="Z22" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA22" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB22" s="2" t="inlineStr"/>
+      <c r="AC22" s="2" t="inlineStr"/>
+      <c r="AD22" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:47:16</t>
+        </is>
+      </c>
+      <c r="AF22" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG22" s="2" t="inlineStr">
+        <is>
+          <t>3999f8b7b140</t>
+        </is>
+      </c>
+      <c r="AH22" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/INVENT Umwelt- und Verfahrenstechnik AG_career.html</t>
+        </is>
+      </c>
+      <c r="AI22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Q-00022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>K7 IT-Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.k7-it.de/willkommen/servicestellen/</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>K7 IT-Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.k7-it.de/</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.k7-it.de/willkommen/servicestellen/</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: K7 IT-Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="inlineStr"/>
+      <c r="X23" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y23" s="2" t="inlineStr">
+        <is>
+          <t>it-</t>
+        </is>
+      </c>
+      <c r="Z23" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA23" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB23" s="2" t="inlineStr"/>
+      <c r="AC23" s="2" t="inlineStr"/>
+      <c r="AD23" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:47:36</t>
+        </is>
+      </c>
+      <c r="AF23" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG23" s="2" t="inlineStr">
+        <is>
+          <t>9970e9fb069b</t>
+        </is>
+      </c>
+      <c r="AH23" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/K7 IT-Solutions GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Q-00023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>K7 Online-Support</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>UX/UI Design</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>K7 Online-Support
+Für schnelle und unmittelbare Unterstützung nutzen Sie bitte den Online-Support der K7-Hotline.
+K7 arbeitet mit den Werkzeugen von „TeamViewer“.
+Klicken Sie auf den nachfolgenden Support-Button, laden Sie die Datei herunter und starten Sie diese. Sie erhalten dann einen Sitzungscode, den Sie der K7-Hotline telefonisch (09131 / 400 33 77) mitteilen.
+&lt;- bitte hier klicken
+Alternativ laden Sie die Quick-Support-Anwendung auf der Teamviewer-Webseite
+mit folgendem Link herunter:
+https://download.teamviewer.com/download/TeamViewerQS.exe
+Alles Weitere klärt der Mitarbeiter der K7-Hotline mit Ihnen.</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.k7-it.de/support/k7-online-support/</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>K7 IT-Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.k7-it.de/</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.k7-it.de/willkommen/servicestellen/</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: K7 IT-Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="inlineStr"/>
+      <c r="X24" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y24" s="2" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="Z24" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA24" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB24" s="2" t="inlineStr"/>
+      <c r="AC24" s="2" t="inlineStr"/>
+      <c r="AD24" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:47:36</t>
+        </is>
+      </c>
+      <c r="AF24" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG24" s="2" t="inlineStr">
+        <is>
+          <t>9970e9fb069b</t>
+        </is>
+      </c>
+      <c r="AH24" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/K7 IT-Solutions GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI24" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/job_detail_v3/job_96866.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Q-00024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Nicolas JamesIT- Beschaffung</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kommunalbit.de/Karriere/</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>KommunalBIT IT-Betreuung Schulen</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kommunalbit.de/</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kommunalbit.de/Karriere/</t>
+        </is>
+      </c>
+      <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U25" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: KommunalBIT IT-Betreuung Schulen</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="inlineStr"/>
+      <c r="X25" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y25" s="2" t="inlineStr">
+        <is>
+          <t>it-</t>
+        </is>
+      </c>
+      <c r="Z25" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA25" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB25" s="2" t="inlineStr"/>
+      <c r="AC25" s="2" t="inlineStr"/>
+      <c r="AD25" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:47:57</t>
+        </is>
+      </c>
+      <c r="AF25" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG25" s="2" t="inlineStr">
+        <is>
+          <t>dd7169947071</t>
+        </is>
+      </c>
+      <c r="AH25" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/KommunalBIT IT-Betreuung Schulen_career.html</t>
+        </is>
+      </c>
+      <c r="AI25" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Junior IT-Jobs quellennah - 36 Jobs (+10)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Quellennah.xlsx
+++ b/download/Junior_IT_Jobs_Quellennah.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI25"/>
+  <dimension ref="A1:AI37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4149,6 +4149,1740 @@
       </c>
       <c r="AI25" s="2" t="inlineStr"/>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Q-00025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung: Elektroniker/in Fachrichtung Energie- und Gebäudetechnik</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>IT-Ausbildung &amp; Studium</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ley-elektrotechnik.de/wir-ueber-uns/stellenangebote.html</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>LEY Elektrotechnik GmbH</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ley-elektrotechnik.de/</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ley-elektrotechnik.de/wir-ueber-uns/stellenangebote.html</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: LEY Elektrotechnik GmbH</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="inlineStr"/>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>ausbildung</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr">
+        <is>
+          <t>elektronik</t>
+        </is>
+      </c>
+      <c r="Z26" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA26" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB26" s="2" t="inlineStr"/>
+      <c r="AC26" s="2" t="inlineStr"/>
+      <c r="AD26" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:54:21</t>
+        </is>
+      </c>
+      <c r="AF26" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG26" s="2" t="inlineStr">
+        <is>
+          <t>28012e2a0bad</t>
+        </is>
+      </c>
+      <c r="AH26" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/LEY Elektrotechnik GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Q-00026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>App Entwickler (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Softwareentwicklung</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>https://profitsoftware.de/jobs.htm</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>ProFit</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>https://profitsoftware.de/</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>https://profitsoftware.de/jobs.htm</t>
+        </is>
+      </c>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: ProFit</t>
+        </is>
+      </c>
+      <c r="W27" s="2" t="inlineStr"/>
+      <c r="X27" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y27" s="2" t="inlineStr">
+        <is>
+          <t>entwickler</t>
+        </is>
+      </c>
+      <c r="Z27" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA27" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB27" s="2" t="inlineStr"/>
+      <c r="AC27" s="2" t="inlineStr"/>
+      <c r="AD27" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:55:15</t>
+        </is>
+      </c>
+      <c r="AF27" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG27" s="2" t="inlineStr">
+        <is>
+          <t>a46ea3afe9b2</t>
+        </is>
+      </c>
+      <c r="AH27" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/ProFit_career.html</t>
+        </is>
+      </c>
+      <c r="AI27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Q-00027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>5★ IT-Bestseller</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.frasch.de/über-uns/karriere/</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>Raphael Frasch GmbH | IT-Systemhaus</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.frasch.de/</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.frasch.de/über-uns/karriere/</t>
+        </is>
+      </c>
+      <c r="S28" s="2" t="inlineStr"/>
+      <c r="T28" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V28" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Raphael Frasch GmbH | IT-Systemhaus</t>
+        </is>
+      </c>
+      <c r="W28" s="2" t="inlineStr"/>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y28" s="2" t="inlineStr">
+        <is>
+          <t>it-</t>
+        </is>
+      </c>
+      <c r="Z28" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA28" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB28" s="2" t="inlineStr"/>
+      <c r="AC28" s="2" t="inlineStr"/>
+      <c r="AD28" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:55:55</t>
+        </is>
+      </c>
+      <c r="AF28" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG28" s="2" t="inlineStr">
+        <is>
+          <t>e576b358abe7</t>
+        </is>
+      </c>
+      <c r="AH28" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Raphael Frasch GmbH _ IT-Systemhaus_career.html</t>
+        </is>
+      </c>
+      <c r="AI28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Q-00028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Azubi Fachinformatiker:in</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>IT-Ausbildung &amp; Studium</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.frasch.de/wir-suchen-sie/azubi-fachinformatiker-in/</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>Raphael Frasch GmbH | IT-Systemhaus</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.frasch.de/</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.frasch.de/über-uns/karriere/</t>
+        </is>
+      </c>
+      <c r="S29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V29" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Raphael Frasch GmbH | IT-Systemhaus</t>
+        </is>
+      </c>
+      <c r="W29" s="2" t="inlineStr"/>
+      <c r="X29" s="2" t="inlineStr">
+        <is>
+          <t>azubi</t>
+        </is>
+      </c>
+      <c r="Y29" s="2" t="inlineStr">
+        <is>
+          <t>informatik</t>
+        </is>
+      </c>
+      <c r="Z29" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA29" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB29" s="2" t="inlineStr"/>
+      <c r="AC29" s="2" t="inlineStr"/>
+      <c r="AD29" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:55:55</t>
+        </is>
+      </c>
+      <c r="AF29" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG29" s="2" t="inlineStr">
+        <is>
+          <t>e576b358abe7</t>
+        </is>
+      </c>
+      <c r="AH29" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Raphael Frasch GmbH _ IT-Systemhaus_career.html</t>
+        </is>
+      </c>
+      <c r="AI29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Q-00029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Netzwerk- und Systemadministrator:in</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Systemadministration</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.frasch.de/wir-suchen-sie/netzwerk-und-systemadministrator-in/</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>Raphael Frasch GmbH | IT-Systemhaus</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.frasch.de/</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.frasch.de/über-uns/karriere/</t>
+        </is>
+      </c>
+      <c r="S30" s="2" t="inlineStr"/>
+      <c r="T30" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Raphael Frasch GmbH | IT-Systemhaus</t>
+        </is>
+      </c>
+      <c r="W30" s="2" t="inlineStr"/>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="inlineStr"/>
+      <c r="AD30" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:55:55</t>
+        </is>
+      </c>
+      <c r="AF30" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG30" s="2" t="inlineStr">
+        <is>
+          <t>e576b358abe7</t>
+        </is>
+      </c>
+      <c r="AH30" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Raphael Frasch GmbH _ IT-Systemhaus_career.html</t>
+        </is>
+      </c>
+      <c r="AI30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Q-00030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>SERVICETECHNIKER (M/W/D) SICHERHEITSTECHNIK</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.janus-sicherheit.de/de/karriere</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>Serity GmbH</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.janus-sicherheit.de/?msclkid=8f8543ca7b0a144234b029cfd9949d66&amp;utm_source=bing&amp;utm_medium=cpc&amp;utm_campaign=1_Unternehmen%20MSP&amp;utm_term=%2BSecurity%20%2BFirma&amp;utm_content=Security</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.janus-sicherheit.de/de/karriere</t>
+        </is>
+      </c>
+      <c r="S31" s="2" t="inlineStr"/>
+      <c r="T31" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Serity GmbH</t>
+        </is>
+      </c>
+      <c r="W31" s="2" t="inlineStr"/>
+      <c r="X31" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y31" s="2" t="inlineStr">
+        <is>
+          <t>sicherheit</t>
+        </is>
+      </c>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB31" s="2" t="inlineStr"/>
+      <c r="AC31" s="2" t="inlineStr"/>
+      <c r="AD31" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:56:33</t>
+        </is>
+      </c>
+      <c r="AF31" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG31" s="2" t="inlineStr">
+        <is>
+          <t>6a13ccc8e82d</t>
+        </is>
+      </c>
+      <c r="AH31" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Serity GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Q-00031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>SERVICETECHNIKER (M/W/D) SICHERHEITSTECHNIK
+– Würzburg</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>#1365
+SERVICETECHNIKER (M/W/D) SICHERHEITSTECHNIK
+Gestalten Sie Ihre Zukunft mit der Janus Sicherheitsdienst GmbH
+Als familiengeführtes Unternehmen mit über 75 Jahren Erfahrung entwickeln wir maßgeschneiderte Sicherheitslösungen für Kunden aus unterschiedlichsten Branchen.
+Zur Verstärkung unseres Teams suchen wir einen Servicetechniker (m/w/d) im Bereich Sicherheitstechnik für den Raum Würzburg.
+Ihr Arbeitsalltag bei uns
+Als Servicetechniker (m/w/d) Sicherheitstechnik sorgen Sie dafür, dass unsere Sicherheitslösungen bei Kunden zuverlässig installiert, gewartet und instand gehalten werden.
+Sie arbeiten praxisnah, lösungsorientiert und an wechselnden Einsatzorten im Raum Würzburg und Umgebung.
+IHRE AUFGABEN
+Planung, Installation und Inbetriebnahme von Sicherheitssystemen (Videoüberwachung, Alarmanlagen)
+Wartung und Instandhaltung bestehender Anlagen
+Analyse und Behebung technischer Störungen vor Ort (regionale Einsätze)
+Einrichtung, Betreuung und Entstörung von Computer-</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.janus-sicherheit.de/de/karriere/servicetechniker-m-w-d-sicherheitstechnik</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr"/>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>Serity GmbH</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.janus-sicherheit.de/?msclkid=8f8543ca7b0a144234b029cfd9949d66&amp;utm_source=bing&amp;utm_medium=cpc&amp;utm_campaign=1_Unternehmen%20MSP&amp;utm_term=%2BSecurity%20%2BFirma&amp;utm_content=Security</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.janus-sicherheit.de/de/karriere</t>
+        </is>
+      </c>
+      <c r="S32" s="2" t="inlineStr"/>
+      <c r="T32" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V32" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Serity GmbH</t>
+        </is>
+      </c>
+      <c r="W32" s="2" t="inlineStr"/>
+      <c r="X32" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y32" s="2" t="inlineStr">
+        <is>
+          <t>sicherheit</t>
+        </is>
+      </c>
+      <c r="Z32" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA32" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB32" s="2" t="inlineStr"/>
+      <c r="AC32" s="2" t="inlineStr"/>
+      <c r="AD32" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:56:33</t>
+        </is>
+      </c>
+      <c r="AF32" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG32" s="2" t="inlineStr">
+        <is>
+          <t>6a13ccc8e82d</t>
+        </is>
+      </c>
+      <c r="AH32" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Serity GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI32" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/job_detail_v3/job_87111.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Q-00032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>SICHERHEITSKRÄFTE (M/W/D) FÜR DIE STADTGALERIE SCHWEINFURT
+– Schweinfurt</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.janus-sicherheit.de/de/karriere/sicherheitskraefte-m-w-d-im-raum-schweinfurt</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>Serity GmbH</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.janus-sicherheit.de/?msclkid=8f8543ca7b0a144234b029cfd9949d66&amp;utm_source=bing&amp;utm_medium=cpc&amp;utm_campaign=1_Unternehmen%20MSP&amp;utm_term=%2BSecurity%20%2BFirma&amp;utm_content=Security</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.janus-sicherheit.de/de/karriere</t>
+        </is>
+      </c>
+      <c r="S33" s="2" t="inlineStr"/>
+      <c r="T33" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V33" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Serity GmbH</t>
+        </is>
+      </c>
+      <c r="W33" s="2" t="inlineStr"/>
+      <c r="X33" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y33" s="2" t="inlineStr">
+        <is>
+          <t>sicherheit</t>
+        </is>
+      </c>
+      <c r="Z33" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA33" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB33" s="2" t="inlineStr"/>
+      <c r="AC33" s="2" t="inlineStr"/>
+      <c r="AD33" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:56:33</t>
+        </is>
+      </c>
+      <c r="AF33" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG33" s="2" t="inlineStr">
+        <is>
+          <t>6a13ccc8e82d</t>
+        </is>
+      </c>
+      <c r="AH33" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Serity GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Q-00033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Field Service Engineering &amp; Customer Service</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com/careers</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr"/>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>Siemens Healthineers</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com/careers</t>
+        </is>
+      </c>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>Medizintechnikhersteller</t>
+        </is>
+      </c>
+      <c r="T34" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V34" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Siemens Healthineers</t>
+        </is>
+      </c>
+      <c r="W34" s="2" t="inlineStr"/>
+      <c r="X34" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y34" s="2" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="Z34" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA34" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB34" s="2" t="inlineStr"/>
+      <c r="AC34" s="2" t="inlineStr"/>
+      <c r="AD34" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:56:41</t>
+        </is>
+      </c>
+      <c r="AF34" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG34" s="2" t="inlineStr">
+        <is>
+          <t>8b145430ddad</t>
+        </is>
+      </c>
+      <c r="AH34" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Siemens Healthineers_career.html</t>
+        </is>
+      </c>
+      <c r="AI34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Q-00034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Support &amp; Dokumentation</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com/deu/careers/faq</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr"/>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="Q35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com/deu</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com/deu/careers/faq</t>
+        </is>
+      </c>
+      <c r="S35" s="2" t="inlineStr">
+        <is>
+          <t>Medizintechnikhersteller</t>
+        </is>
+      </c>
+      <c r="T35" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U35" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V35" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="W35" s="2" t="inlineStr"/>
+      <c r="X35" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y35" s="2" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="Z35" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA35" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB35" s="2" t="inlineStr"/>
+      <c r="AC35" s="2" t="inlineStr"/>
+      <c r="AD35" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:56:50</t>
+        </is>
+      </c>
+      <c r="AF35" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG35" s="2" t="inlineStr">
+        <is>
+          <t>bf046f872f92</t>
+        </is>
+      </c>
+      <c r="AH35" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/Siemens Healthineers AG_career.html</t>
+        </is>
+      </c>
+      <c r="AI35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Q-00035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Projektleiter Elektrotechnik (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>https://tks-service.de/de/karriere/</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>TKS Datentechnik GmbH</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>https://tks-service.de/de/dienstleistungen/datentechnik</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>https://tks-service.de/de/karriere/</t>
+        </is>
+      </c>
+      <c r="S36" s="2" t="inlineStr">
+        <is>
+          <t>IT-Berater</t>
+        </is>
+      </c>
+      <c r="T36" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V36" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: TKS Datentechnik GmbH</t>
+        </is>
+      </c>
+      <c r="W36" s="2" t="inlineStr"/>
+      <c r="X36" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y36" s="2" t="inlineStr">
+        <is>
+          <t>elektrotechnik</t>
+        </is>
+      </c>
+      <c r="Z36" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA36" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB36" s="2" t="inlineStr"/>
+      <c r="AC36" s="2" t="inlineStr"/>
+      <c r="AD36" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:57:19</t>
+        </is>
+      </c>
+      <c r="AF36" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG36" s="2" t="inlineStr">
+        <is>
+          <t>858dc152173a</t>
+        </is>
+      </c>
+      <c r="AH36" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/TKS Datentechnik GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Q-00036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>IT-Visionär(innen) und Vertriebs-Enthusiast(inn)en</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>https://tribar.de/karriere/</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr"/>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>TRIBAR Software GmbH</t>
+        </is>
+      </c>
+      <c r="Q37" s="2" t="inlineStr">
+        <is>
+          <t>https://tribar.de/</t>
+        </is>
+      </c>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>https://tribar.de/karriere/</t>
+        </is>
+      </c>
+      <c r="S37" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T37" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U37" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V37" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: TRIBAR Software GmbH</t>
+        </is>
+      </c>
+      <c r="W37" s="2" t="inlineStr"/>
+      <c r="X37" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y37" s="2" t="inlineStr">
+        <is>
+          <t>it-</t>
+        </is>
+      </c>
+      <c r="Z37" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA37" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB37" s="2" t="inlineStr"/>
+      <c r="AC37" s="2" t="inlineStr"/>
+      <c r="AD37" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE37" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:57:32</t>
+        </is>
+      </c>
+      <c r="AF37" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG37" s="2" t="inlineStr">
+        <is>
+          <t>41619367fd5c</t>
+        </is>
+      </c>
+      <c r="AH37" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/TRIBAR Software GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI37" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Junior IT-Jobs quellennah - 52 Jobs (+11)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Quellennah.xlsx
+++ b/download/Junior_IT_Jobs_Quellennah.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI37"/>
+  <dimension ref="A1:AI53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5883,6 +5883,2354 @@
       </c>
       <c r="AI37" s="2" t="inlineStr"/>
     </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Q-00037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>An engineering technician working at a lab.</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ul.com/careers</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>UL Solutions</t>
+        </is>
+      </c>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>https://germany.ul.com/en/locations/</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ul.com/careers</t>
+        </is>
+      </c>
+      <c r="S38" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T38" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V38" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: UL Solutions</t>
+        </is>
+      </c>
+      <c r="W38" s="2" t="inlineStr"/>
+      <c r="X38" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y38" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z38" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA38" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB38" s="2" t="inlineStr"/>
+      <c r="AC38" s="2" t="inlineStr"/>
+      <c r="AD38" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE38" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:59:35</t>
+        </is>
+      </c>
+      <c r="AF38" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG38" s="2" t="inlineStr">
+        <is>
+          <t>1e32dec11cf9</t>
+        </is>
+      </c>
+      <c r="AH38" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/UL Solutions_career.html</t>
+        </is>
+      </c>
+      <c r="AI38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Q-00038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Plastics and Engineered Materials</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Cyber Security</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>As a global safety science leader, UL Solutions helps companies to demonstrate safety, enhance sustainability, strengthen security, deliver quality, manage risk and achieve regulatory compliance.</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ul.com/industries/chemicals-and-materials/plastics-and-engineered-materials</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr"/>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>UL Solutions</t>
+        </is>
+      </c>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>https://germany.ul.com/en/locations/</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ul.com/careers</t>
+        </is>
+      </c>
+      <c r="S39" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T39" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U39" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V39" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: UL Solutions</t>
+        </is>
+      </c>
+      <c r="W39" s="2" t="inlineStr"/>
+      <c r="X39" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y39" s="2" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="Z39" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA39" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB39" s="2" t="inlineStr"/>
+      <c r="AC39" s="2" t="inlineStr"/>
+      <c r="AD39" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE39" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:59:35</t>
+        </is>
+      </c>
+      <c r="AF39" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG39" s="2" t="inlineStr">
+        <is>
+          <t>1e32dec11cf9</t>
+        </is>
+      </c>
+      <c r="AH39" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/UL Solutions_career.html</t>
+        </is>
+      </c>
+      <c r="AI39" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/job_detail_v3/job_35063.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Q-00039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Services</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ul.com/sis/engineering</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr"/>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>UL Solutions</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>https://germany.ul.com/en/locations/</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ul.com/careers</t>
+        </is>
+      </c>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V40" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: UL Solutions</t>
+        </is>
+      </c>
+      <c r="W40" s="2" t="inlineStr"/>
+      <c r="X40" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y40" s="2" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="Z40" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA40" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB40" s="2" t="inlineStr"/>
+      <c r="AC40" s="2" t="inlineStr"/>
+      <c r="AD40" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE40" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:59:35</t>
+        </is>
+      </c>
+      <c r="AF40" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG40" s="2" t="inlineStr">
+        <is>
+          <t>1e32dec11cf9</t>
+        </is>
+      </c>
+      <c r="AH40" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/UL Solutions_career.html</t>
+        </is>
+      </c>
+      <c r="AI40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Q-00040</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Engineering process management</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ul.com/sis/stages/engineering-process-management</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr"/>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>UL Solutions</t>
+        </is>
+      </c>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t>https://germany.ul.com/en/locations/</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ul.com/careers</t>
+        </is>
+      </c>
+      <c r="S41" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T41" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U41" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V41" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: UL Solutions</t>
+        </is>
+      </c>
+      <c r="W41" s="2" t="inlineStr"/>
+      <c r="X41" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y41" s="2" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="Z41" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA41" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB41" s="2" t="inlineStr"/>
+      <c r="AC41" s="2" t="inlineStr"/>
+      <c r="AD41" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE41" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:59:35</t>
+        </is>
+      </c>
+      <c r="AF41" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG41" s="2" t="inlineStr">
+        <is>
+          <t>1e32dec11cf9</t>
+        </is>
+      </c>
+      <c r="AH41" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/UL Solutions_career.html</t>
+        </is>
+      </c>
+      <c r="AI41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Q-00041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Energy
+    Software tools and data support for developing, assessing and operating renewable energy projects.</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ul.com/software/ultrus/energy</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr"/>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>UL Solutions</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>https://germany.ul.com/en/locations/</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ul.com/careers</t>
+        </is>
+      </c>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V42" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: UL Solutions</t>
+        </is>
+      </c>
+      <c r="W42" s="2" t="inlineStr"/>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y42" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z42" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA42" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB42" s="2" t="inlineStr"/>
+      <c r="AC42" s="2" t="inlineStr"/>
+      <c r="AD42" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE42" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:59:35</t>
+        </is>
+      </c>
+      <c r="AF42" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG42" s="2" t="inlineStr">
+        <is>
+          <t>1e32dec11cf9</t>
+        </is>
+      </c>
+      <c r="AH42" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/UL Solutions_career.html</t>
+        </is>
+      </c>
+      <c r="AI42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Q-00042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Du liebst Technik, IT-Infrastrukturen und smarte Lösungen? Du möchtest nicht nur Probleme erkennen, sondern sie aktiv lösen? Dann bist du bei uns genau richtig!</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bitma.de/team/karriere.html</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr"/>
+      <c r="O43" s="2" t="inlineStr"/>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>bITma solutions GmbH</t>
+        </is>
+      </c>
+      <c r="Q43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bitma.de/</t>
+        </is>
+      </c>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bitma.de/team/karriere.html</t>
+        </is>
+      </c>
+      <c r="S43" s="2" t="inlineStr"/>
+      <c r="T43" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U43" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V43" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: bITma solutions GmbH</t>
+        </is>
+      </c>
+      <c r="W43" s="2" t="inlineStr"/>
+      <c r="X43" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y43" s="2" t="inlineStr">
+        <is>
+          <t>it-</t>
+        </is>
+      </c>
+      <c r="Z43" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA43" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB43" s="2" t="inlineStr"/>
+      <c r="AC43" s="2" t="inlineStr"/>
+      <c r="AD43" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE43" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:01:16</t>
+        </is>
+      </c>
+      <c r="AF43" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG43" s="2" t="inlineStr">
+        <is>
+          <t>afcc3abe9fcb</t>
+        </is>
+      </c>
+      <c r="AH43" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/bITma solutions GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Q-00043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Software-Entwickler (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Softwareentwicklung</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.emesit.net/jobs.php</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr"/>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>emesit Innovative Maschinen und Software</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.emesit.net/kontakt.php</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.emesit.net/jobs.php</t>
+        </is>
+      </c>
+      <c r="S44" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T44" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V44" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: emesit Innovative Maschinen und Software</t>
+        </is>
+      </c>
+      <c r="W44" s="2" t="inlineStr"/>
+      <c r="X44" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y44" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z44" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA44" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB44" s="2" t="inlineStr"/>
+      <c r="AC44" s="2" t="inlineStr"/>
+      <c r="AD44" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE44" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:01:52</t>
+        </is>
+      </c>
+      <c r="AF44" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG44" s="2" t="inlineStr">
+        <is>
+          <t>bd73b6b57b9c</t>
+        </is>
+      </c>
+      <c r="AH44" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/emesit Innovative Maschinen und Software_career.html</t>
+        </is>
+      </c>
+      <c r="AI44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Q-00044</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Architekt*in Wohnungsbau (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr"/>
+      <c r="O45" s="2" t="inlineStr"/>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="Q45" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/kontakt/kontaktdaten/</t>
+        </is>
+      </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/</t>
+        </is>
+      </c>
+      <c r="S45" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T45" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U45" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V45" s="2" t="inlineStr">
+        <is>
+          <t>nav_footer: ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="W45" s="2" t="inlineStr"/>
+      <c r="X45" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y45" s="2" t="inlineStr">
+        <is>
+          <t>architekt</t>
+        </is>
+      </c>
+      <c r="Z45" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA45" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB45" s="2" t="inlineStr"/>
+      <c r="AC45" s="2" t="inlineStr"/>
+      <c r="AD45" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE45" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:02:04</t>
+        </is>
+      </c>
+      <c r="AF45" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG45" s="2" t="inlineStr">
+        <is>
+          <t>0d11239631dd</t>
+        </is>
+      </c>
+      <c r="AH45" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/ercas Software Solutions GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Q-00045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Architekt*in Wohnungsbau (m/w/d)
+Vollzeit in Nürnberg
+Kategorie: Technisch</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>DevOps &amp; Cloud</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zurück zu allen Positionen
+Architekt*in Wohnungsbau (m/w/d)
+Beschäftigungsart
+Festanstellung, Vollzeit
+Arbeitsort
+Nürnberg
+Berufserfahrung
+mind. 5 Jahre
+Ihre Aufgaben
+Eigenständige Erarbeitung und Erstellung von Planungsunterlagen über alle Projektphasen hinweg.
+Verantwortliche Prüfung und Sicherstellung der Konformität von Planunterlagen mit Gesetzen, Normen und Richtlinien.
+Übernahme hoher Verantwortung bei der Steuerung von Großprojekten von Anfang an.
+Aktive Mitarbeit an der Digitalisierung von Bauprozessen (z.B. BIM, TEAM3 + etc.).
+Sicheres und kommunikationsstarkes Auftreten im Umgang mit externen Partnern wie Bauherren und Behörden.
+Vertretung des Projekts in Abstimmungsgesprächen und bei Genehmigungsverfahren.
+Ihr Profil
+Erfolgreich abgeschlossenes Hochschulstudium (z.B. Dipl.-Ing., Master oder vergleichbar) im relevanten technischen oder planerischen Bereich.
+Tiefe Kenntnisse in den Bereichen Bau- und Planungsrecht, Bautechnik und Projektmanagement.
+Umfassendes Wissen </t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/job-architekt-in-wohnungsbau-m-w-d-nuernberg-3676</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr"/>
+      <c r="O46" s="2" t="inlineStr"/>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/kontakt/kontaktdaten/</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T46" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U46" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V46" s="2" t="inlineStr">
+        <is>
+          <t>nav_footer: ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="W46" s="2" t="inlineStr"/>
+      <c r="X46" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y46" s="2" t="inlineStr">
+        <is>
+          <t>architekt</t>
+        </is>
+      </c>
+      <c r="Z46" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA46" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB46" s="2" t="inlineStr"/>
+      <c r="AC46" s="2" t="inlineStr"/>
+      <c r="AD46" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE46" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:02:04</t>
+        </is>
+      </c>
+      <c r="AF46" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG46" s="2" t="inlineStr">
+        <is>
+          <t>0d11239631dd</t>
+        </is>
+      </c>
+      <c r="AH46" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/ercas Software Solutions GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI46" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/job_detail_v3/job_20547.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Q-00046</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>IT-Netzwerkspezialist im nationalen und internationalen IT-Support (m/w/d)
+Vollzeit in Erlangen
+Kategorie: Technisch</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/job-it-netzwerkspezialist-im-nationalen-und-internationalen-it-support-m-w-d-erlangen-3664</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr"/>
+      <c r="O47" s="2" t="inlineStr"/>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="Q47" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/kontakt/kontaktdaten/</t>
+        </is>
+      </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/</t>
+        </is>
+      </c>
+      <c r="S47" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T47" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U47" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V47" s="2" t="inlineStr">
+        <is>
+          <t>nav_footer: ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="W47" s="2" t="inlineStr"/>
+      <c r="X47" s="2" t="inlineStr">
+        <is>
+          <t>intern</t>
+        </is>
+      </c>
+      <c r="Y47" s="2" t="inlineStr">
+        <is>
+          <t>it-</t>
+        </is>
+      </c>
+      <c r="Z47" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA47" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB47" s="2" t="inlineStr"/>
+      <c r="AC47" s="2" t="inlineStr"/>
+      <c r="AD47" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE47" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:02:04</t>
+        </is>
+      </c>
+      <c r="AF47" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG47" s="2" t="inlineStr">
+        <is>
+          <t>0d11239631dd</t>
+        </is>
+      </c>
+      <c r="AH47" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/ercas Software Solutions GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Q-00047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Our work combines deep expertise in radar and simulation with modern software engineering and scalable compute infrastructure. We collaborate closely with industry partners and work on real-world projects in automotive, aerospace, and more.</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Softwareentwicklung</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>https://fived.ai/careers</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr"/>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>fiveD GmbH</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="inlineStr">
+        <is>
+          <t>https://fived.ai/</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>https://fived.ai/careers</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T48" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U48" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V48" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: fiveD GmbH</t>
+        </is>
+      </c>
+      <c r="W48" s="2" t="inlineStr"/>
+      <c r="X48" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y48" s="2" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+      <c r="Z48" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA48" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB48" s="2" t="inlineStr"/>
+      <c r="AC48" s="2" t="inlineStr"/>
+      <c r="AD48" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE48" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:02:15</t>
+        </is>
+      </c>
+      <c r="AF48" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG48" s="2" t="inlineStr">
+        <is>
+          <t>bf55037cafe2</t>
+        </is>
+      </c>
+      <c r="AH48" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/fiveD GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Q-00048</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>’As a consultant and chief engineer at infoteam, I have the opportunity to work on the front line on many current industry topics such as Big Data and Industry 4.0.’</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>https://infoteam.de/en/career-at-infoteam</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr"/>
+      <c r="O49" s="2" t="inlineStr"/>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>infoteam Software AG</t>
+        </is>
+      </c>
+      <c r="Q49" s="2" t="inlineStr">
+        <is>
+          <t>https://infoteam.de/en</t>
+        </is>
+      </c>
+      <c r="R49" s="2" t="inlineStr">
+        <is>
+          <t>https://infoteam.de/en/career-at-infoteam</t>
+        </is>
+      </c>
+      <c r="S49" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T49" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U49" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V49" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: infoteam Software AG</t>
+        </is>
+      </c>
+      <c r="W49" s="2" t="inlineStr"/>
+      <c r="X49" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y49" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="Z49" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA49" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB49" s="2" t="inlineStr"/>
+      <c r="AC49" s="2" t="inlineStr"/>
+      <c r="AD49" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE49" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:02:23</t>
+        </is>
+      </c>
+      <c r="AF49" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG49" s="2" t="inlineStr">
+        <is>
+          <t>02eab742c816</t>
+        </is>
+      </c>
+      <c r="AH49" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/infoteam Software AG_career.html</t>
+        </is>
+      </c>
+      <c r="AI49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Q-00049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>New trainees on board
+09/04/2023 | Career news 09/04/2023 | Corporate</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>IT-Ausbildung &amp; Studium</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Trainee</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>https://infoteam.de/en/news-1/detail/neue-azubis-an-bord</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr"/>
+      <c r="O50" s="2" t="inlineStr"/>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>infoteam Software AG</t>
+        </is>
+      </c>
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>https://infoteam.de/en</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>https://infoteam.de/en/career-at-infoteam</t>
+        </is>
+      </c>
+      <c r="S50" s="2" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="T50" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U50" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V50" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: infoteam Software AG</t>
+        </is>
+      </c>
+      <c r="W50" s="2" t="inlineStr"/>
+      <c r="X50" s="2" t="inlineStr">
+        <is>
+          <t>trainee</t>
+        </is>
+      </c>
+      <c r="Y50" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z50" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA50" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB50" s="2" t="inlineStr"/>
+      <c r="AC50" s="2" t="inlineStr"/>
+      <c r="AD50" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE50" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:02:23</t>
+        </is>
+      </c>
+      <c r="AF50" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG50" s="2" t="inlineStr">
+        <is>
+          <t>02eab742c816</t>
+        </is>
+      </c>
+      <c r="AH50" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/infoteam Software AG_career.html</t>
+        </is>
+      </c>
+      <c r="AI50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Q-00050</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Bewirb Dich über unsere Website, WhatsApp, Social Media oder auf diversen Stellenportalen – mit oder ohne Lebenslauf.</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>https://karriere-bei.persona.de/?utm_source=persona.de&amp;utm_medium=footer&amp;utm_campaign=footer</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr"/>
+      <c r="O51" s="2" t="inlineStr"/>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>persona service AG &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="Q51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.persona.de/en-gb/location/erlangen</t>
+        </is>
+      </c>
+      <c r="R51" s="2" t="inlineStr">
+        <is>
+          <t>https://karriere-bei.persona.de/?utm_source=persona.de&amp;utm_medium=footer&amp;utm_campaign=footer</t>
+        </is>
+      </c>
+      <c r="S51" s="2" t="inlineStr">
+        <is>
+          <t>Zeitarbeitsagentur</t>
+        </is>
+      </c>
+      <c r="T51" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U51" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V51" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: persona service AG &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="W51" s="2" t="inlineStr"/>
+      <c r="X51" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y51" s="2" t="inlineStr">
+        <is>
+          <t>sap</t>
+        </is>
+      </c>
+      <c r="Z51" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA51" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB51" s="2" t="inlineStr"/>
+      <c r="AC51" s="2" t="inlineStr"/>
+      <c r="AD51" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE51" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:02:35</t>
+        </is>
+      </c>
+      <c r="AF51" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG51" s="2" t="inlineStr">
+        <is>
+          <t>23c4f0d60a10</t>
+        </is>
+      </c>
+      <c r="AH51" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/persona service AG _ Co. KG_career.html</t>
+        </is>
+      </c>
+      <c r="AI51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Q-00051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>schmidt IT ist ein führendes IT-Systemhaus mit Fokus auf IT-Sicherheit, IT-Infrastruktur und IT-Support. Seit 2001 sind wir in der Metropolregion Nürnberg-Erlangen-Fürth für Unternehmen und Organisationen erfolgreich tätig.</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Cyber Security</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.msit-gmbh.de/karriere-bei-msit/</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr"/>
+      <c r="O52" s="2" t="inlineStr"/>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>schmidt IT GmbH</t>
+        </is>
+      </c>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.msit-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="R52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.msit-gmbh.de/karriere-bei-msit/</t>
+        </is>
+      </c>
+      <c r="S52" s="2" t="inlineStr"/>
+      <c r="T52" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U52" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V52" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: schmidt IT GmbH</t>
+        </is>
+      </c>
+      <c r="W52" s="2" t="inlineStr"/>
+      <c r="X52" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y52" s="2" t="inlineStr">
+        <is>
+          <t>it-</t>
+        </is>
+      </c>
+      <c r="Z52" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA52" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB52" s="2" t="inlineStr"/>
+      <c r="AC52" s="2" t="inlineStr"/>
+      <c r="AD52" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE52" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:02:43</t>
+        </is>
+      </c>
+      <c r="AF52" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG52" s="2" t="inlineStr">
+        <is>
+          <t>d748f6838686</t>
+        </is>
+      </c>
+      <c r="AH52" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/schmidt IT GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Q-00052</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft – Support</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.msit-gmbh.de/microsoft-support/</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>Metropolregion Nürnberg (Kern)</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr"/>
+      <c r="O53" s="2" t="inlineStr"/>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>schmidt IT GmbH</t>
+        </is>
+      </c>
+      <c r="Q53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.msit-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="R53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.msit-gmbh.de/karriere-bei-msit/</t>
+        </is>
+      </c>
+      <c r="S53" s="2" t="inlineStr"/>
+      <c r="T53" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U53" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V53" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: schmidt IT GmbH</t>
+        </is>
+      </c>
+      <c r="W53" s="2" t="inlineStr"/>
+      <c r="X53" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y53" s="2" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="Z53" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA53" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB53" s="2" t="inlineStr"/>
+      <c r="AC53" s="2" t="inlineStr"/>
+      <c r="AD53" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE53" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:02:43</t>
+        </is>
+      </c>
+      <c r="AF53" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG53" s="2" t="inlineStr">
+        <is>
+          <t>d748f6838686</t>
+        </is>
+      </c>
+      <c r="AH53" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/schmidt IT GmbH_career.html</t>
+        </is>
+      </c>
+      <c r="AI53" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Junior IT-Jobs quellennah - 62 Jobs (+10)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Quellennah.xlsx
+++ b/download/Junior_IT_Jobs_Quellennah.xlsx
@@ -435,8 +435,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI53"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:AI63"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -8231,6 +8231,1526 @@
       </c>
       <c r="AI53" s="2" t="inlineStr"/>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Q-00053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Öko-Modellregion freut sich über neue Abholstellen für Gemüse-Abokisten</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.100prozentbamberg.de/news/umwelt/oeko-modellregion-freut-sich-ueber-neue-abholstellen-fuer-gemuese-abokisten</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr"/>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>100% Bamberg e.K.</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.100prozentbamberg.de</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.100prozentbamberg.de/news/umwelt/oeko-modellregion-freut-sich-ueber-neue-abholstellen-fuer-gemuese-abokisten</t>
+        </is>
+      </c>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V54" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: 100% Bamberg e.K.</t>
+        </is>
+      </c>
+      <c r="W54" s="2" t="inlineStr"/>
+      <c r="X54" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y54" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="Z54" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA54" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB54" s="2" t="inlineStr"/>
+      <c r="AC54" s="2" t="inlineStr"/>
+      <c r="AD54" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE54" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:03:20</t>
+        </is>
+      </c>
+      <c r="AF54" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG54" s="2" t="inlineStr">
+        <is>
+          <t>d1b3a411ae71</t>
+        </is>
+      </c>
+      <c r="AH54" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/100_ Bamberg e.K_career.html</t>
+        </is>
+      </c>
+      <c r="AI54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Q-00054</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>ESSO Tankstelle Hirschaid</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.100prozentbamberg.de/tankstelle/esso-tankstelle-hirschaid</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr"/>
+      <c r="O55" s="2" t="inlineStr"/>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>100% Bamberg e.K.</t>
+        </is>
+      </c>
+      <c r="Q55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.100prozentbamberg.de</t>
+        </is>
+      </c>
+      <c r="R55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.100prozentbamberg.de/news/umwelt/oeko-modellregion-freut-sich-ueber-neue-abholstellen-fuer-gemuese-abokisten</t>
+        </is>
+      </c>
+      <c r="S55" s="2" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="T55" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U55" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V55" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: 100% Bamberg e.K.</t>
+        </is>
+      </c>
+      <c r="W55" s="2" t="inlineStr"/>
+      <c r="X55" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y55" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z55" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA55" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB55" s="2" t="inlineStr"/>
+      <c r="AC55" s="2" t="inlineStr"/>
+      <c r="AD55" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE55" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:03:20</t>
+        </is>
+      </c>
+      <c r="AF55" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG55" s="2" t="inlineStr">
+        <is>
+          <t>d1b3a411ae71</t>
+        </is>
+      </c>
+      <c r="AH55" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/100_ Bamberg e.K_career.html</t>
+        </is>
+      </c>
+      <c r="AI55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Q-00055</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>b&amp;p engineering mobility GmbH</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.100prozentbamberg.de/handwerk-und-industrie-in-bamberg/bp-engineering-mobility-gmbh</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr"/>
+      <c r="O56" s="2" t="inlineStr"/>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>100% Bamberg e.K.</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.100prozentbamberg.de</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.100prozentbamberg.de/news/umwelt/oeko-modellregion-freut-sich-ueber-neue-abholstellen-fuer-gemuese-abokisten</t>
+        </is>
+      </c>
+      <c r="S56" s="2" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="T56" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U56" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: 100% Bamberg e.K.</t>
+        </is>
+      </c>
+      <c r="W56" s="2" t="inlineStr"/>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y56" s="2" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="Z56" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA56" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB56" s="2" t="inlineStr"/>
+      <c r="AC56" s="2" t="inlineStr"/>
+      <c r="AD56" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE56" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:03:20</t>
+        </is>
+      </c>
+      <c r="AF56" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG56" s="2" t="inlineStr">
+        <is>
+          <t>d1b3a411ae71</t>
+        </is>
+      </c>
+      <c r="AH56" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/100_ Bamberg e.K_career.html</t>
+        </is>
+      </c>
+      <c r="AI56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Q-00056</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Interne Trainer &amp; Experten</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr"/>
+      <c r="O57" s="2" t="inlineStr"/>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="Q57" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/standort/bamberg-arwa/498</t>
+        </is>
+      </c>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa</t>
+        </is>
+      </c>
+      <c r="S57" s="2" t="inlineStr">
+        <is>
+          <t>dienstleistung</t>
+        </is>
+      </c>
+      <c r="T57" s="2" t="inlineStr">
+        <is>
+          <t>Website (Text)</t>
+        </is>
+      </c>
+      <c r="U57" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V57" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="W57" s="2" t="inlineStr"/>
+      <c r="X57" s="2" t="inlineStr">
+        <is>
+          <t>intern</t>
+        </is>
+      </c>
+      <c r="Y57" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z57" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA57" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB57" s="2" t="inlineStr"/>
+      <c r="AC57" s="2" t="inlineStr"/>
+      <c r="AD57" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE57" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:03:38</t>
+        </is>
+      </c>
+      <c r="AF57" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG57" s="2" t="inlineStr">
+        <is>
+          <t>7c338217b1bd</t>
+        </is>
+      </c>
+      <c r="AH57" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/ARWA Personaldienstleistungen GmbH - Bamberg_career.html</t>
+        </is>
+      </c>
+      <c r="AI57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Q-00057</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>NEU
+Personaldisponent (m/w/d)
+ARWA-Ludwigsfelde
+STANDORT
+14974 Ludwigsfelde
+ARBEITSZEIT
+Vollzeit
+Details ansehen</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Wir bei ARWA Personaldienstleistungen GmbH suchen für unseren internen Bereich einen zuverlässigen &lt;strong&gt;Personaldisponent (m/w/d)&lt;/strong&gt; in &lt;strong&gt;Ludwigsfelde&lt;/strong&gt;, der die &lt;strong&gt;strategische Planung und Koordination unserer Personalressourcen&lt;/strong&gt; übernimmt und als &lt;strong&gt;zentrale Schnittstelle&lt;/strong&gt; zwischen unseren Kunden und Bewerbern fungiert.&lt;br&gt;&lt;br /&gt;Mit Ihrem &lt;strong&gt;ausgeprägten organisatorischen Talent&lt;/strong&gt; und Ihrer &lt;strong&gt;überzeugenden Kommunikationsstärke&lt;/strong&gt; sorgen Sie für die optimale Besetzung offener Stellen und den reibungslosen Personaleinsatz.&lt;br&lt;br /&gt;Diese verantwortungsvolle Position bieten wir Ihnen in &lt;strong&gt;Vollzeit&lt;/strong&gt; an.&lt;/p&gt;&lt;br /&gt;&lt;br /&gt;&lt;h3&gt;Vorteile, die Ihnen zugutekommen&lt;/h3&gt;&lt;br /&gt;&lt;ul&gt;&lt;br /&gt;  &lt;li&gt;Betriebsarzt/Betriebsärztin&lt;/li&gt;&lt;br /&gt;&lt;li&gt;Flache Hierarchien&lt;/li&gt;&lt;br /&gt;&lt;li&gt;Kostenlose Getränke&lt;/li&gt;&lt;br /&gt;&lt;/ul&gt;&lt;br /&gt;&lt;br /&gt;&lt;h3&gt;Ihre Aufgaben auf einen Blick&lt;/h3&gt;&lt;br /&gt;&lt;ul&gt;&lt;br /&gt;  &lt;li&gt;Sie verantworten die aktive Neukundengewinn</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa/job/2199/personaldisponent-ludwigsfelde/</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr"/>
+      <c r="O58" s="2" t="inlineStr"/>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/standort/bamberg-arwa/498</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa</t>
+        </is>
+      </c>
+      <c r="S58" s="2" t="inlineStr">
+        <is>
+          <t>dienstleistung</t>
+        </is>
+      </c>
+      <c r="T58" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U58" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V58" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="W58" s="2" t="inlineStr"/>
+      <c r="X58" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y58" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z58" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA58" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB58" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="AC58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD58" s="2" t="inlineStr">
+        <is>
+          <t>Frisch (≤ 7 Tage)</t>
+        </is>
+      </c>
+      <c r="AE58" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:03:38</t>
+        </is>
+      </c>
+      <c r="AF58" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG58" s="2" t="inlineStr">
+        <is>
+          <t>7c338217b1bd</t>
+        </is>
+      </c>
+      <c r="AH58" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/ARWA Personaldienstleistungen GmbH - Bamberg_career.html</t>
+        </is>
+      </c>
+      <c r="AI58" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/job_detail_v3/job_22997.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Q-00058</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>NEU
+Personaldisponent (m/w/d)
+ARWA-Salzwedel
+STANDORT
+29410 Salzwedel
+ARBEITSZEIT
+Vollzeit
+Details ansehen</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>UX/UI Design</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Wir bei ARWA Personaldienstleistungen GmbH suchen für unseren internen Bereich einen zuverlässigen &lt;strong&gt;Personaldisponent (m/w/d)&lt;/strong&gt; in &lt;strong&gt;Salzwedel&lt;/strong&gt;, der die &lt;strong&gt;strategische Planung und Koordination unserer Personalressourcen&lt;/strong&gt; übernimmt und als &lt;strong&gt;zentrale Schnittstelle&lt;/strong&gt; zwischen unseren Kunden und Bewerbern fungiert.&lt;br&gt;&lt;br /&gt;Mit Ihrem &lt;strong&gt;ausgeprägten organisatorischen Talent&lt;/strong&gt; und Ihrer &lt;strong&gt;überzeugenden Kommunikationsstärke&lt;/strong&gt; sorgen Sie für die optimale Besetzung offener Stellen und den reibungslosen Personaleinsatz.&lt;br&lt;br /&gt;Diese verantwortungsvolle Position bieten wir Ihnen in &lt;strong&gt;Vollzeit&lt;/strong&gt; an.&lt;/p&gt;&lt;br /&gt;&lt;br /&gt;&lt;h3&gt;Vorteile, die Ihnen zugutekommen&lt;/h3&gt;&lt;br /&gt;&lt;ul&gt;&lt;br /&gt;  &lt;li&gt;Betriebsarzt/Betriebsärztin&lt;/li&gt;&lt;br /&gt;&lt;li&gt;Digitales Onboarding im Unternehmen&lt;/li&gt;&lt;br /&gt;&lt;li&gt;Kostenlose Getränke&lt;/li&gt;&lt;br /&gt;&lt;li&gt;Preisnachlässe auf Produkte/Dienstleistungen&lt;/li&gt;&lt;br /&gt;&lt;/ul&gt;&lt;br /&gt;&lt;br /&gt;&lt;h3&gt;Ihre Aufgaben auf einen Bl</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa/job/2198/personaldisponent-salzwedel/</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr"/>
+      <c r="O59" s="2" t="inlineStr"/>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="Q59" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/standort/bamberg-arwa/498</t>
+        </is>
+      </c>
+      <c r="R59" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa</t>
+        </is>
+      </c>
+      <c r="S59" s="2" t="inlineStr">
+        <is>
+          <t>dienstleistung</t>
+        </is>
+      </c>
+      <c r="T59" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U59" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V59" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="W59" s="2" t="inlineStr"/>
+      <c r="X59" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y59" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z59" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA59" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB59" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="AC59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD59" s="2" t="inlineStr">
+        <is>
+          <t>Frisch (≤ 7 Tage)</t>
+        </is>
+      </c>
+      <c r="AE59" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:03:38</t>
+        </is>
+      </c>
+      <c r="AF59" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG59" s="2" t="inlineStr">
+        <is>
+          <t>7c338217b1bd</t>
+        </is>
+      </c>
+      <c r="AH59" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/ARWA Personaldienstleistungen GmbH - Bamberg_career.html</t>
+        </is>
+      </c>
+      <c r="AI59" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/job_detail_v3/job_53895.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Q-00059</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>NEU
+Personaldisponent - Quereinsteiger (m/w/d)
+ARWA-Bayreuth
+STANDORT
+95444 Bayreuth
+ARBEITSZEIT
+Vollzeit
+Details ansehen</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Berufseinsteiger</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa/job/2197/personaldisponent-quereinsteiger-bayreuth/</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr"/>
+      <c r="O60" s="2" t="inlineStr"/>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/standort/bamberg-arwa/498</t>
+        </is>
+      </c>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa</t>
+        </is>
+      </c>
+      <c r="S60" s="2" t="inlineStr">
+        <is>
+          <t>dienstleistung</t>
+        </is>
+      </c>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U60" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V60" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="W60" s="2" t="inlineStr"/>
+      <c r="X60" s="2" t="inlineStr">
+        <is>
+          <t>einsteiger</t>
+        </is>
+      </c>
+      <c r="Y60" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z60" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA60" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB60" s="2" t="inlineStr"/>
+      <c r="AC60" s="2" t="inlineStr"/>
+      <c r="AD60" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE60" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:03:38</t>
+        </is>
+      </c>
+      <c r="AF60" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG60" s="2" t="inlineStr">
+        <is>
+          <t>7c338217b1bd</t>
+        </is>
+      </c>
+      <c r="AH60" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/ARWA Personaldienstleistungen GmbH - Bamberg_career.html</t>
+        </is>
+      </c>
+      <c r="AI60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Q-00060</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>NEU
+Personaldisponent - Quereinsteiger (m/w/d)
+ARWA-Oldenburg
+STANDORT
+26122 Oldenburg
+ARBEITSZEIT
+Vollzeit
+Details ansehen</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Berufseinsteiger</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa/job/2196/personaldisponent-quereinsteiger-oldenburg/</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr"/>
+      <c r="O61" s="2" t="inlineStr"/>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="Q61" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/standort/bamberg-arwa/498</t>
+        </is>
+      </c>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa</t>
+        </is>
+      </c>
+      <c r="S61" s="2" t="inlineStr">
+        <is>
+          <t>dienstleistung</t>
+        </is>
+      </c>
+      <c r="T61" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U61" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V61" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="W61" s="2" t="inlineStr"/>
+      <c r="X61" s="2" t="inlineStr">
+        <is>
+          <t>einsteiger</t>
+        </is>
+      </c>
+      <c r="Y61" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z61" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA61" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB61" s="2" t="inlineStr"/>
+      <c r="AC61" s="2" t="inlineStr"/>
+      <c r="AD61" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE61" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:03:38</t>
+        </is>
+      </c>
+      <c r="AF61" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG61" s="2" t="inlineStr">
+        <is>
+          <t>7c338217b1bd</t>
+        </is>
+      </c>
+      <c r="AH61" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/ARWA Personaldienstleistungen GmbH - Bamberg_career.html</t>
+        </is>
+      </c>
+      <c r="AI61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Q-00061</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>NEU
+Personaldisponent (m/w/d)
+ARWA-Oldenburg
+STANDORT
+26122 Oldenburg
+ARBEITSZEIT
+Vollzeit
+Details ansehen</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Junior-fähig</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa/job/2195/personaldisponent-oldenburg/</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr"/>
+      <c r="O62" s="2" t="inlineStr"/>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/standort/bamberg-arwa/498</t>
+        </is>
+      </c>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa</t>
+        </is>
+      </c>
+      <c r="S62" s="2" t="inlineStr">
+        <is>
+          <t>dienstleistung</t>
+        </is>
+      </c>
+      <c r="T62" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U62" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V62" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="W62" s="2" t="inlineStr"/>
+      <c r="X62" s="2" t="inlineStr">
+        <is>
+          <t>no_senior_keyword</t>
+        </is>
+      </c>
+      <c r="Y62" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z62" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA62" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB62" s="2" t="inlineStr"/>
+      <c r="AC62" s="2" t="inlineStr"/>
+      <c r="AD62" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE62" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:03:38</t>
+        </is>
+      </c>
+      <c r="AF62" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG62" s="2" t="inlineStr">
+        <is>
+          <t>7c338217b1bd</t>
+        </is>
+      </c>
+      <c r="AH62" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/ARWA Personaldienstleistungen GmbH - Bamberg_career.html</t>
+        </is>
+      </c>
+      <c r="AI62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Q-00062</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>NEU
+Personaldisponent - Quereinsteiger (m/w/d)
+ARWA-Hamburg
+STANDORT
+20095 Hamburg
+ARBEITSZEIT
+Vollzeit
+Details ansehen</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>IT (Sonstige)</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Berufseinsteiger</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Vollzeit</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Nicht angegeben</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa/job/2194/personaldisponent-quereinsteiger-hamburg/</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>Oberfranken</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr"/>
+      <c r="O63" s="2" t="inlineStr"/>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/standort/bamberg-arwa/498</t>
+        </is>
+      </c>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t>https://arwa.de/de/ueber-arwa/karriere-bei-arwa</t>
+        </is>
+      </c>
+      <c r="S63" s="2" t="inlineStr">
+        <is>
+          <t>dienstleistung</t>
+        </is>
+      </c>
+      <c r="T63" s="2" t="inlineStr">
+        <is>
+          <t>Website (Link)</t>
+        </is>
+      </c>
+      <c r="U63" s="2" t="inlineStr">
+        <is>
+          <t>Website direkt</t>
+        </is>
+      </c>
+      <c r="V63" s="2" t="inlineStr">
+        <is>
+          <t>website_navigation: ARWA Personaldienstleistungen GmbH - Bamberg</t>
+        </is>
+      </c>
+      <c r="W63" s="2" t="inlineStr"/>
+      <c r="X63" s="2" t="inlineStr">
+        <is>
+          <t>einsteiger</t>
+        </is>
+      </c>
+      <c r="Y63" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="Z63" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AA63" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="AB63" s="2" t="inlineStr"/>
+      <c r="AC63" s="2" t="inlineStr"/>
+      <c r="AD63" s="2" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="AE63" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14 19:03:38</t>
+        </is>
+      </c>
+      <c r="AF63" s="2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="AG63" s="2" t="inlineStr">
+        <is>
+          <t>7c338217b1bd</t>
+        </is>
+      </c>
+      <c r="AH63" s="2" t="inlineStr">
+        <is>
+          <t>/home/z/my-project/download/career_pages_v3/ARWA Personaldienstleistungen GmbH - Bamberg_career.html</t>
+        </is>
+      </c>
+      <c r="AI63" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Junior IT-Jobs quellennah - 119 Jobs (+8)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Quellennah.xlsx
+++ b/download/Junior_IT_Jobs_Quellennah.xlsx
@@ -16662,7 +16662,7 @@
       </c>
       <c r="AE110" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:52:00</t>
+          <t>2026-05-14 19:52:23</t>
         </is>
       </c>
       <c r="AF110" s="2" t="inlineStr">
@@ -16682,7 +16682,7 @@
       </c>
       <c r="AI110" s="2" t="inlineStr">
         <is>
-          <t>/home/z/my-project/download/job_detail_v3/job_11263.html</t>
+          <t>/home/z/my-project/download/job_detail_v3/job_64097.html</t>
         </is>
       </c>
     </row>
@@ -16807,7 +16807,7 @@
       </c>
       <c r="AE111" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:52:07</t>
+          <t>2026-05-14 19:52:29</t>
         </is>
       </c>
       <c r="AF111" s="2" t="inlineStr">
@@ -16948,7 +16948,7 @@
       </c>
       <c r="AE112" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:52:17</t>
+          <t>2026-05-14 19:52:38</t>
         </is>
       </c>
       <c r="AF112" s="2" t="inlineStr">
@@ -17093,7 +17093,7 @@
       </c>
       <c r="AE113" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:54:16</t>
+          <t>2026-05-14 19:54:35</t>
         </is>
       </c>
       <c r="AF113" s="2" t="inlineStr">
@@ -17234,7 +17234,7 @@
       </c>
       <c r="AE114" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:55:12</t>
+          <t>2026-05-14 19:55:31</t>
         </is>
       </c>
       <c r="AF114" s="2" t="inlineStr">
@@ -17375,7 +17375,7 @@
       </c>
       <c r="AE115" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:55:21</t>
+          <t>2026-05-14 19:55:40</t>
         </is>
       </c>
       <c r="AF115" s="2" t="inlineStr">
@@ -17516,7 +17516,7 @@
       </c>
       <c r="AE116" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:55:35</t>
+          <t>2026-05-14 19:55:56</t>
         </is>
       </c>
       <c r="AF116" s="2" t="inlineStr">
@@ -17657,7 +17657,7 @@
       </c>
       <c r="AE117" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:56:30</t>
+          <t>2026-05-14 19:56:34</t>
         </is>
       </c>
       <c r="AF117" s="2" t="inlineStr">
@@ -17801,7 +17801,7 @@
       </c>
       <c r="AE118" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:56:30</t>
+          <t>2026-05-14 19:56:34</t>
         </is>
       </c>
       <c r="AF118" s="2" t="inlineStr">
@@ -17945,7 +17945,7 @@
       </c>
       <c r="AE119" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:56:30</t>
+          <t>2026-05-14 19:56:34</t>
         </is>
       </c>
       <c r="AF119" s="2" t="inlineStr">
@@ -18089,7 +18089,7 @@
       </c>
       <c r="AE120" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:56:30</t>
+          <t>2026-05-14 19:56:34</t>
         </is>
       </c>
       <c r="AF120" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Junior IT-Jobs quellennah - 119 Jobs (+4)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Quellennah.xlsx
+++ b/download/Junior_IT_Jobs_Quellennah.xlsx
@@ -17657,7 +17657,7 @@
       </c>
       <c r="AE117" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:56:34</t>
+          <t>2026-05-14 19:56:35</t>
         </is>
       </c>
       <c r="AF117" s="2" t="inlineStr">
@@ -17801,7 +17801,7 @@
       </c>
       <c r="AE118" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:56:34</t>
+          <t>2026-05-14 19:56:35</t>
         </is>
       </c>
       <c r="AF118" s="2" t="inlineStr">
@@ -17945,7 +17945,7 @@
       </c>
       <c r="AE119" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:56:34</t>
+          <t>2026-05-14 19:56:35</t>
         </is>
       </c>
       <c r="AF119" s="2" t="inlineStr">
@@ -18089,7 +18089,7 @@
       </c>
       <c r="AE120" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:56:34</t>
+          <t>2026-05-14 19:56:35</t>
         </is>
       </c>
       <c r="AF120" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Junior IT-Jobs quellennah - 119 Jobs (+7)
</commit_message>
<xml_diff>
--- a/download/Junior_IT_Jobs_Quellennah.xlsx
+++ b/download/Junior_IT_Jobs_Quellennah.xlsx
@@ -17234,7 +17234,7 @@
       </c>
       <c r="AE114" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:55:31</t>
+          <t>2026-05-14 19:55:38</t>
         </is>
       </c>
       <c r="AF114" s="2" t="inlineStr">
@@ -17375,7 +17375,7 @@
       </c>
       <c r="AE115" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:55:40</t>
+          <t>2026-05-14 19:55:45</t>
         </is>
       </c>
       <c r="AF115" s="2" t="inlineStr">
@@ -17516,7 +17516,7 @@
       </c>
       <c r="AE116" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:55:56</t>
+          <t>2026-05-14 19:55:59</t>
         </is>
       </c>
       <c r="AF116" s="2" t="inlineStr">
@@ -17657,7 +17657,7 @@
       </c>
       <c r="AE117" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:56:35</t>
+          <t>2026-05-14 19:56:39</t>
         </is>
       </c>
       <c r="AF117" s="2" t="inlineStr">
@@ -17801,7 +17801,7 @@
       </c>
       <c r="AE118" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:56:35</t>
+          <t>2026-05-14 19:56:39</t>
         </is>
       </c>
       <c r="AF118" s="2" t="inlineStr">
@@ -17945,7 +17945,7 @@
       </c>
       <c r="AE119" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:56:35</t>
+          <t>2026-05-14 19:56:39</t>
         </is>
       </c>
       <c r="AF119" s="2" t="inlineStr">
@@ -18089,7 +18089,7 @@
       </c>
       <c r="AE120" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14 19:56:35</t>
+          <t>2026-05-14 19:56:39</t>
         </is>
       </c>
       <c r="AF120" s="2" t="inlineStr">

</xml_diff>